<commit_message>
Final data input data
</commit_message>
<xml_diff>
--- a/Data Input/099_2024_tagData.xlsx
+++ b/Data Input/099_2024_tagData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://instreamf.sharepoint.com/sites/099-BulkleySK/Shared Documents/3 - Analyses/2024_R/099_Bulkley_Telem_2024/Data Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{F090F347-808B-48AF-8FE4-E896DD36E23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1572B99-03EF-48B9-B328-91875F0C4FDE}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{F090F347-808B-48AF-8FE4-E896DD36E23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09459755-A488-4520-A51A-9A5823118067}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{97613F0C-1A42-4FAB-A3B6-C30F5CC1359E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{97613F0C-1A42-4FAB-A3B6-C30F5CC1359E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -574,7 +574,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2776C8A4-916A-4D06-A5D3-9D7E739280E9}" name="Table2" displayName="Table2" ref="A1:K173" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:K173" xr:uid="{2776C8A4-916A-4D06-A5D3-9D7E739280E9}"/>
+  <autoFilter ref="A1:K173" xr:uid="{2776C8A4-916A-4D06-A5D3-9D7E739280E9}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Seine"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K173">
     <sortCondition ref="B1:B173"/>
   </sortState>
@@ -961,7 +967,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6">
         <v>45485</v>
       </c>
@@ -985,7 +991,7 @@
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6">
         <v>45485</v>
       </c>
@@ -1009,7 +1015,7 @@
       </c>
       <c r="H3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="6">
         <v>45488</v>
       </c>
@@ -1033,7 +1039,7 @@
       </c>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6">
         <v>45488</v>
       </c>
@@ -1060,7 +1066,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6">
         <v>45488</v>
       </c>
@@ -1084,7 +1090,7 @@
       </c>
       <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
         <v>45488</v>
       </c>
@@ -1108,7 +1114,7 @@
       </c>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <v>45489</v>
       </c>
@@ -1132,7 +1138,7 @@
       </c>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
         <v>45488</v>
       </c>
@@ -1156,7 +1162,7 @@
       </c>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <v>45489</v>
       </c>
@@ -1180,7 +1186,7 @@
       </c>
       <c r="H10" s="3"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <v>45489</v>
       </c>
@@ -1426,7 +1432,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
         <v>45490</v>
       </c>
@@ -1450,7 +1456,7 @@
       </c>
       <c r="H22" s="3"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6">
         <v>45490</v>
       </c>
@@ -1474,7 +1480,7 @@
       </c>
       <c r="H23" s="3"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6">
         <v>45490</v>
       </c>
@@ -1498,7 +1504,7 @@
       </c>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6">
         <v>45490</v>
       </c>
@@ -1522,7 +1528,7 @@
       </c>
       <c r="H25" s="3"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6">
         <v>45490</v>
       </c>
@@ -1546,7 +1552,7 @@
       </c>
       <c r="H26" s="3"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6">
         <v>45490</v>
       </c>
@@ -1570,7 +1576,7 @@
       </c>
       <c r="H27" s="3"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
         <v>45490</v>
       </c>
@@ -1594,7 +1600,7 @@
       </c>
       <c r="H28" s="3"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6">
         <v>45491</v>
       </c>
@@ -1618,7 +1624,7 @@
       </c>
       <c r="H29" s="3"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="6">
         <v>45491</v>
       </c>
@@ -1642,7 +1648,7 @@
       </c>
       <c r="H30" s="3"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6">
         <v>45491</v>
       </c>
@@ -1666,7 +1672,7 @@
       </c>
       <c r="H31" s="3"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6">
         <v>45491</v>
       </c>
@@ -1690,7 +1696,7 @@
       </c>
       <c r="H32" s="3"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6">
         <v>45491</v>
       </c>
@@ -1714,7 +1720,7 @@
       </c>
       <c r="H33" s="3"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
         <v>45491</v>
       </c>
@@ -1738,7 +1744,7 @@
       </c>
       <c r="H34" s="3"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6">
         <v>45491</v>
       </c>
@@ -1762,7 +1768,7 @@
       </c>
       <c r="H35" s="3"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
         <v>45491</v>
       </c>
@@ -1786,7 +1792,7 @@
       </c>
       <c r="H36" s="3"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6">
         <v>45491</v>
       </c>
@@ -1810,7 +1816,7 @@
       </c>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6">
         <v>45491</v>
       </c>
@@ -1834,7 +1840,7 @@
       </c>
       <c r="H38" s="3"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6">
         <v>45491</v>
       </c>
@@ -1858,7 +1864,7 @@
       </c>
       <c r="H39" s="3"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6">
         <v>45491</v>
       </c>
@@ -1882,7 +1888,7 @@
       </c>
       <c r="H40" s="3"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6">
         <v>45491</v>
       </c>
@@ -1906,7 +1912,7 @@
       </c>
       <c r="H41" s="3"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6">
         <v>45492</v>
       </c>
@@ -1930,7 +1936,7 @@
       </c>
       <c r="H42" s="3"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6">
         <v>45492</v>
       </c>
@@ -1954,7 +1960,7 @@
       </c>
       <c r="H43" s="3"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6">
         <v>45492</v>
       </c>
@@ -1978,7 +1984,7 @@
       </c>
       <c r="H44" s="3"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6">
         <v>45492</v>
       </c>
@@ -2005,7 +2011,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6">
         <v>45492</v>
       </c>
@@ -2032,7 +2038,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6">
         <v>45492</v>
       </c>
@@ -2059,7 +2065,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="6">
         <v>45495</v>
       </c>
@@ -2083,7 +2089,7 @@
       </c>
       <c r="H48" s="3"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6">
         <v>45495</v>
       </c>
@@ -2107,7 +2113,7 @@
       </c>
       <c r="H49" s="3"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="6">
         <v>45495</v>
       </c>
@@ -2131,7 +2137,7 @@
       </c>
       <c r="H50" s="3"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6">
         <v>45495</v>
       </c>
@@ -2395,7 +2401,7 @@
       </c>
       <c r="H61" s="3"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="6">
         <v>45495</v>
       </c>
@@ -2419,7 +2425,7 @@
       </c>
       <c r="H62" s="3"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="6">
         <v>45495</v>
       </c>
@@ -2443,7 +2449,7 @@
       </c>
       <c r="H63" s="3"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6">
         <v>45495</v>
       </c>
@@ -2467,7 +2473,7 @@
       </c>
       <c r="H64" s="3"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="6">
         <v>45495</v>
       </c>
@@ -2491,7 +2497,7 @@
       </c>
       <c r="H65" s="3"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="6">
         <v>45495</v>
       </c>
@@ -2515,7 +2521,7 @@
       </c>
       <c r="H66" s="3"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="6">
         <v>45495</v>
       </c>
@@ -2539,7 +2545,7 @@
       </c>
       <c r="H67" s="3"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="6">
         <v>45496</v>
       </c>
@@ -2563,7 +2569,7 @@
       </c>
       <c r="H68" s="3"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="6">
         <v>45496</v>
       </c>
@@ -2587,7 +2593,7 @@
       </c>
       <c r="H69" s="3"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="6">
         <v>45496</v>
       </c>
@@ -2611,7 +2617,7 @@
       </c>
       <c r="H70" s="3"/>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="6">
         <v>45496</v>
       </c>
@@ -3182,7 +3188,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="6">
         <v>45496</v>
       </c>
@@ -3211,7 +3217,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="6">
         <v>45496</v>
       </c>
@@ -3240,7 +3246,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="6">
         <v>45496</v>
       </c>
@@ -3267,7 +3273,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="6">
         <v>45496</v>
       </c>
@@ -3296,7 +3302,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="6">
         <v>45497</v>
       </c>
@@ -3325,7 +3331,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="6">
         <v>45497</v>
       </c>
@@ -3354,7 +3360,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="6">
         <v>45497</v>
       </c>
@@ -3383,7 +3389,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="6">
         <v>45497</v>
       </c>
@@ -3412,7 +3418,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="6">
         <v>45498</v>
       </c>
@@ -3441,7 +3447,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="6">
         <v>45498</v>
       </c>
@@ -3470,7 +3476,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="6">
         <v>45498</v>
       </c>
@@ -3499,7 +3505,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="6">
         <v>45498</v>
       </c>
@@ -3528,7 +3534,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="6">
         <v>45499</v>
       </c>
@@ -3557,7 +3563,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="6">
         <v>45502</v>
       </c>
@@ -3586,7 +3592,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="6">
         <v>45502</v>
       </c>
@@ -3615,7 +3621,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="6">
         <v>45503</v>
       </c>
@@ -3644,7 +3650,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="6">
         <v>45504</v>
       </c>
@@ -3673,7 +3679,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="6">
         <v>45504</v>
       </c>
@@ -3702,7 +3708,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="6">
         <v>45504</v>
       </c>
@@ -3731,7 +3737,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="6">
         <v>45504</v>
       </c>
@@ -3876,7 +3882,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="6">
         <v>45505</v>
       </c>
@@ -3905,7 +3911,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="6">
         <v>45505</v>
       </c>
@@ -3934,7 +3940,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="6">
         <v>45505</v>
       </c>
@@ -3963,7 +3969,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="6">
         <v>45505</v>
       </c>
@@ -3990,7 +3996,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="6">
         <v>45505</v>
       </c>
@@ -4019,7 +4025,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="6">
         <v>45505</v>
       </c>
@@ -4048,7 +4054,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="6">
         <v>45505</v>
       </c>
@@ -4077,7 +4083,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="6">
         <v>45505</v>
       </c>
@@ -4101,7 +4107,7 @@
       </c>
       <c r="H122" s="3"/>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="6">
         <v>45505</v>
       </c>
@@ -4130,7 +4136,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="6">
         <v>45505</v>
       </c>
@@ -4159,7 +4165,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="6">
         <v>45505</v>
       </c>
@@ -4188,7 +4194,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="6">
         <v>45505</v>
       </c>
@@ -4217,7 +4223,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="6">
         <v>45505</v>
       </c>
@@ -4246,7 +4252,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="6">
         <v>45505</v>
       </c>
@@ -4391,7 +4397,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="6">
         <v>45512</v>
       </c>
@@ -4420,7 +4426,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="6">
         <v>45512</v>
       </c>
@@ -4623,7 +4629,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="6">
         <v>45512</v>
       </c>
@@ -4647,7 +4653,7 @@
       </c>
       <c r="H141" s="3"/>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="6">
         <v>45512</v>
       </c>
@@ -4671,7 +4677,7 @@
       </c>
       <c r="H142" s="3"/>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="6">
         <v>45512</v>
       </c>
@@ -4700,7 +4706,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="6">
         <v>45512</v>
       </c>
@@ -4729,7 +4735,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="6">
         <v>45512</v>
       </c>
@@ -4758,7 +4764,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="6">
         <v>45512</v>
       </c>
@@ -4787,7 +4793,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="6">
         <v>45512</v>
       </c>
@@ -4816,7 +4822,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="6">
         <v>45512</v>
       </c>
@@ -5106,7 +5112,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="6">
         <v>45498</v>
       </c>
@@ -5130,7 +5136,7 @@
       </c>
       <c r="H158" s="3"/>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="6">
         <v>45498</v>
       </c>
@@ -5154,7 +5160,7 @@
       </c>
       <c r="H159" s="3"/>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="6">
         <v>45498</v>
       </c>
@@ -5178,7 +5184,7 @@
       </c>
       <c r="H160" s="3"/>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" s="6">
         <v>45498</v>
       </c>
@@ -5482,7 +5488,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" s="6">
         <v>45506</v>
       </c>
@@ -5511,7 +5517,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="6">
         <v>45506</v>
       </c>
@@ -5549,6 +5555,29 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="3a1d4ae3-9824-4bd0-a876-bc5475db720a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <DocType xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127" xsi:nil="true"/>
+    <Info xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127" xsi:nil="true"/>
+    <Year xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E81916CCB1D67B4598C0FB6F15BA745D" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8ed6e656783e9961ccc8ccd6cb8c565c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3a1d4ae3-9824-4bd0-a876-bc5475db720a" xmlns:ns3="e6aff03f-7bcb-4894-a843-93db8e1be127" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dbb610e4e8be73c95ee4c551e6fee17" ns2:_="" ns3:_="">
     <xsd:import namespace="3a1d4ae3-9824-4bd0-a876-bc5475db720a"/>
@@ -5823,30 +5852,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B40A2C96-7A63-4DE6-82F7-845F36D99580}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3a1d4ae3-9824-4bd0-a876-bc5475db720a"/>
+    <ds:schemaRef ds:uri="e6aff03f-7bcb-4894-a843-93db8e1be127"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="3a1d4ae3-9824-4bd0-a876-bc5475db720a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <DocType xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127" xsi:nil="true"/>
-    <Info xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127" xsi:nil="true"/>
-    <Year xmlns="e6aff03f-7bcb-4894-a843-93db8e1be127" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{193BCA9E-850B-4CB4-BEA3-863D0C3B221F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9887868C-FE6B-49AC-B988-01593AF87F35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5863,23 +5888,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{193BCA9E-850B-4CB4-BEA3-863D0C3B221F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B40A2C96-7A63-4DE6-82F7-845F36D99580}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3a1d4ae3-9824-4bd0-a876-bc5475db720a"/>
-    <ds:schemaRef ds:uri="e6aff03f-7bcb-4894-a843-93db8e1be127"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>